<commit_message>
M2.5 T1: rebuild raw template with passage-per-row + text ChapterID
</commit_message>
<xml_diff>
--- a/content-pipeline/templates/Raw_Input_template.xlsx
+++ b/content-pipeline/templates/Raw_Input_template.xlsx
@@ -62,10 +62,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -152,7 +156,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Two-digit chapter number, e.g., 01, 02, ..., 20. Determines JSON filename and audio folder.</t>
+        <t>Two-digit chapter number as TEXT, e.g., 00, 01, 02, ..., 20. Cell is formatted as text so leading zeros are preserved. Determines JSON filename (chapterXX.json) and audio folder (audio/chapterXX/).</t>
       </text>
     </comment>
     <comment ref="A3" authorId="0" shapeId="0">
@@ -172,7 +176,9 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>PASSAGE column. Paste your Traditional Chinese passage(s) here. You can spread across multiple rows or all in one cell - Python joins them. Punctuation matters: sentences will be split by 。！？</t>
+        <t>PASSAGE column.
+One passage per row.
+If a passage contains multiple paragraphs, use Alt+Enter INSIDE the same cell to create paragraph breaks. Each Alt+Enter becomes a \n in the JSON. Each row becomes a separate entry in the passages array.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -478,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -503,6 +509,7 @@
           <t>ChapterID</t>
         </is>
       </c>
+      <c r="B2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -510,6 +517,55 @@
           <t>ChapterTitle</t>
         </is>
       </c>
+      <c r="B3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -523,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -547,6 +603,150 @@
           <t>English</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -560,14 +760,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>DFSNMGCSEChinese - Raw Input Template</t>
         </is>
@@ -577,7 +777,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>HOW TO FILL IN THIS TEMPLATE</t>
         </is>
@@ -606,82 +806,94 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2. Meta sheet: Fill in ChapterID (e.g., 01) and ChapterTitle</t>
+          <t>2. Meta sheet:</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - ChapterID: two-digit text, e.g. 00, 01, 02, ...</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3. Content sheet - three independent columns:</t>
+          <t xml:space="preserve">     (Cell B2 is text-formatted so leading zeros are preserved.)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Column A (Passage): Paste your Chinese passage(s). Multiple rows OK.</t>
+          <t xml:space="preserve">   - ChapterTitle: title shown in the app dashboard.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Column B (Vocabulary): Chinese words separated by | (pipe). Multiple rows OK.</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Column C (English): English meanings separated by | (pipe), same order as B.</t>
+          <t>3. Content sheet - three independent columns:</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Column A (Passage):</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4. IMPORTANT: The total count of items in B and C must match.</t>
+          <t xml:space="preserve">     - ONE PASSAGE PER ROW.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Python will error clearly if counts don't align.</t>
+          <t xml:space="preserve">     - If a passage has multiple paragraphs, use Alt+Enter INSIDE the</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       same cell to create paragraph breaks.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5. Upload this file to your Codespace at:</t>
+          <t xml:space="preserve">     - Each row becomes a separate entry in the JSON passages array.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   content-pipeline/inputs/chapterXX_raw.xlsx</t>
+          <t xml:space="preserve">     - Alt+Enter breaks become \n in the JSON.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Column B (Vocabulary): Chinese words separated by | (pipe). Multiple rows OK.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6. Run: python content-pipeline/generate_review.py --input inputs/chapterXX_raw.xlsx</t>
+          <t xml:space="preserve">   Column C (English): English meanings separated by | (pipe), same order as B.</t>
         </is>
       </c>
     </row>
@@ -691,14 +903,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7. Download the generated chapterXX_review.xlsx, check the auto-generated pinyin</t>
+          <t>4. IMPORTANT: The total count of items in B and C must match.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   and context sentences, correct any errors, save as chapterXX_final.xlsx</t>
+          <t xml:space="preserve">   Python will error clearly if counts don't align.</t>
         </is>
       </c>
     </row>
@@ -708,88 +920,211 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8. Upload chapterXX_final.xlsx back to Codespace, then run publish script.</t>
+          <t>5. Upload this file to your Codespace at:</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   content-pipeline/inputs/chapterXX_raw.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>DELIMITER RULE</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Use | (pipe character) to separate items in Vocabulary and English columns.</t>
+          <t>6. Run: python content-pipeline/generate_review.py --input inputs/chapterXX_raw.xlsx</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Do NOT use commas - some English meanings naturally contain commas.</t>
-        </is>
-      </c>
+      <c r="A30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Example: park, garden|to like, prefer  &lt;- would break if using comma delimiter</t>
+          <t>7. Download the generated chapterXX_review.xlsx, check the auto-generated pinyin</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   and context sentences, correct any errors, save as chapterXX_final.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>MULTI-PRONUNCIATION CHARACTERS (多音字)</t>
-        </is>
-      </c>
+      <c r="A33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Some Traditional Chinese characters have multiple pronunciations that pypinyin</t>
+          <t>8. Upload chapterXX_final.xlsx back to Codespace, then run publish script:</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>may guess incorrectly. Common examples:</t>
+          <t xml:space="preserve">   python content-pipeline/generate_chapter.py --input inputs/chapterXX_final.xlsx</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  長: cháng (long) vs zhǎng (elder/grow) - e.g., 長方形 should be cháng fāng xíng</t>
-        </is>
-      </c>
+      <c r="A36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  行: xíng (walk) vs háng (row/profession) - e.g., 銀行 = yín háng</t>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>PASSAGE STRUCTURE EXAMPLES</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  樂: lè (happy) vs yuè (music) - e.g., 音樂 = yīn yuè</t>
+          <t>Example A - single passage, single paragraph:</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Row 2, Column A: 英華國際學校創建於1990年，設有小學和中學。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Example B - single passage, multiple paragraphs (use Alt+Enter):</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Row 2, Column A: 英華國際學校創建於1990年。[Alt+Enter]雙語是這個學校的教學特色。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Example C - multiple passages:</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Row 2, Column A: First passage text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Row 3, Column A: Second passage text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Row 4, Column A: Third passage text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>DELIMITER RULE (Vocabulary + English columns)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Use | (pipe character) to separate items in Vocabulary and English columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Do NOT use commas - some English meanings naturally contain commas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Example: park, garden|to like, prefer  &lt;- would break if using comma delimiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>MULTI-PRONUNCIATION CHARACTERS (多音字)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Some Traditional Chinese characters have multiple pronunciations that pypinyin</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>may guess incorrectly. Common examples:</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  長: cháng (long) vs zhǎng (elder/grow) - e.g., 長方形 should be cháng fāng xíng</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  行: xíng (walk) vs háng (row/profession) - e.g., 銀行 = yín háng</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  樂: lè (happy) vs yuè (music) - e.g., 音樂 = yīn yuè</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>Fix these manually during the review step.</t>
         </is>

</xml_diff>

<commit_message>
M8.3c-1: Multi-book pipeline support with bilingual audio. New generate_common.py with LANGUAGES config (Mandarin Xiaoxiao + Cantonese WanLung, both -10%). BookID validation across 5 layers. Nested audio JSON schema. Old app unchanged.
</commit_message>
<xml_diff>
--- a/content-pipeline/templates/Raw_Input_template.xlsx
+++ b/content-pipeline/templates/Raw_Input_template.xlsx
@@ -156,10 +156,15 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Two-digit chapter number as TEXT, e.g., 00, 01, 02, ..., 20. Cell is formatted as text so leading zeros are preserved. Determines JSON filename (chapterXX.json) and audio folder (audio/chapterXX/).</t>
+        <t>Two-digit book number as TEXT, e.g., 01, 02, 03, ... Cell is formatted as text so leading zeros are preserved. Book must first be registered in data/books-index.json. Determines output folder (data/bookXX/) and audio folder (audio/bookXX/chapterYY/).</t>
       </text>
     </comment>
     <comment ref="A3" authorId="0" shapeId="0">
+      <text>
+        <t>Two-digit chapter number as TEXT, e.g., 01, 02, 03, ... Cell is formatted as text so leading zeros are preserved. Chapter numbers restart at 01 within each book.</t>
+      </text>
+    </comment>
+    <comment ref="A4" authorId="0" shapeId="0">
       <text>
         <t>Chapter title in Chinese or English. Shown in the app dashboard.</t>
       </text>
@@ -506,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ChapterID</t>
+          <t>BookID</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
@@ -514,13 +519,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>ChapterID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>ChapterTitle</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="B4" s="2" t="n"/>
+      <c r="B4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="B5" s="2" t="n"/>
@@ -760,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A60"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -789,14 +799,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1. Save this file as: chapterXX_raw.xlsx (replace XX with chapter number)</t>
+          <t>1. Save this file as: bXX_chYY_raw.xlsx (XX=book number, YY=chapter number)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Example: chapter01_raw.xlsx</t>
+          <t xml:space="preserve">   Example: b01_ch01_raw.xlsx</t>
         </is>
       </c>
     </row>
@@ -813,7 +823,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - ChapterID: two-digit text, e.g. 00, 01, 02, ...</t>
+          <t xml:space="preserve">   - BookID: two-digit text, e.g. 01, 02, 03, ...</t>
         </is>
       </c>
     </row>
@@ -827,90 +837,94 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - ChapterTitle: title shown in the app dashboard.</t>
+          <t xml:space="preserve">     Book must first be registered in data/books-index.json.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - ChapterID: two-digit text, e.g. 01, 02, 03, ...</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3. Content sheet - three independent columns:</t>
+          <t xml:space="preserve">     Chapter numbers restart at 01 within each book.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Column A (Passage):</t>
+          <t xml:space="preserve">   - ChapterTitle: title shown in the app dashboard.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     - ONE PASSAGE PER ROW.</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - If a passage has multiple paragraphs, use Alt+Enter INSIDE the</t>
+          <t>3. Content sheet - three independent columns:</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">       same cell to create paragraph breaks.</t>
+          <t xml:space="preserve">   Column A (Passage):</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - Each row becomes a separate entry in the JSON passages array.</t>
+          <t xml:space="preserve">     - ONE PASSAGE PER ROW.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - Alt+Enter breaks become \n in the JSON.</t>
+          <t xml:space="preserve">     - If a passage has multiple paragraphs, use Alt+Enter INSIDE the</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Column B (Vocabulary): Chinese words separated by | (pipe). Multiple rows OK.</t>
+          <t xml:space="preserve">       same cell to create paragraph breaks.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Column C (English): English meanings separated by | (pipe), same order as B.</t>
+          <t xml:space="preserve">     - Each row becomes a separate entry in the JSON passages array.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     - Alt+Enter breaks become \n in the JSON.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4. IMPORTANT: The total count of items in B and C must match.</t>
+          <t xml:space="preserve">   Column B (Vocabulary): Chinese words separated by | (pipe). Multiple rows OK.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Python will error clearly if counts don't align.</t>
+          <t xml:space="preserve">   Column C (English): English meanings separated by | (pipe), same order as B.</t>
         </is>
       </c>
     </row>
@@ -920,14 +934,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5. Upload this file to your Codespace at:</t>
+          <t>4. IMPORTANT: The total count of items in B and C must match.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">   content-pipeline/inputs/chapterXX_raw.xlsx</t>
+          <t xml:space="preserve">   Python will error clearly if counts don't align.</t>
         </is>
       </c>
     </row>
@@ -937,24 +951,24 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6. Run: python content-pipeline/generate_review.py --input inputs/chapterXX_raw.xlsx</t>
+          <t>5. Upload this file to your Codespace at:</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   content-pipeline/inputs/bookXX/bXX_chYY_raw.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>7. Download the generated chapterXX_review.xlsx, check the auto-generated pinyin</t>
-        </is>
-      </c>
+      <c r="A31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">   and context sentences, correct any errors, save as chapterXX_final.xlsx</t>
+          <t>6. Run: python content-pipeline/generate_review.py --input inputs/bookXX/bXX_chYY_raw.xlsx</t>
         </is>
       </c>
     </row>
@@ -964,14 +978,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>8. Upload chapterXX_final.xlsx back to Codespace, then run publish script:</t>
+          <t>7. Download the generated bXX_chYY_review.xlsx, check the auto-generated pinyin</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   python content-pipeline/generate_chapter.py --input inputs/chapterXX_final.xlsx</t>
+          <t xml:space="preserve">   and context sentences, correct any errors, save as bXX_chYY_final.xlsx</t>
         </is>
       </c>
     </row>
@@ -979,23 +993,23 @@
       <c r="A36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>PASSAGE STRUCTURE EXAMPLES</t>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>8. Upload bXX_chYY_final.xlsx back to Codespace, then run publish script:</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Example A - single passage, single paragraph:</t>
+          <t xml:space="preserve">   python content-pipeline/generate_chapter.py --input inputs/bookXX/bXX_chYY_final.xlsx</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Row 2, Column A: 英華國際學校創建於1990年，設有小學和中學。</t>
+          <t xml:space="preserve">   (Generates 4 MP3s per word: Mandarin + Cantonese, isolated + sentence.)</t>
         </is>
       </c>
     </row>
@@ -1003,128 +1017,152 @@
       <c r="A40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Example B - single passage, multiple paragraphs (use Alt+Enter):</t>
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>PASSAGE STRUCTURE EXAMPLES</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Row 2, Column A: 英華國際學校創建於1990年。[Alt+Enter]雙語是這個學校的教學特色。</t>
+          <t>Example A - single passage, single paragraph:</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Row 2, Column A: 英華國際學校創建於1990年，設有小學和中學。</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Example C - multiple passages:</t>
-        </is>
-      </c>
+      <c r="A44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Row 2, Column A: First passage text.</t>
+          <t>Example B - single passage, multiple paragraphs (use Alt+Enter):</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Row 3, Column A: Second passage text.</t>
+          <t xml:space="preserve">   Row 2, Column A: 英華國際學校創建於1990年。[Alt+Enter]雙語是這個學校的教學特色。</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Row 4, Column A: Third passage text.</t>
-        </is>
-      </c>
+      <c r="A47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Example C - multiple passages:</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>DELIMITER RULE (Vocabulary + English columns)</t>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Row 2, Column A: First passage text.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Use | (pipe character) to separate items in Vocabulary and English columns.</t>
+          <t xml:space="preserve">   Row 3, Column A: Second passage text.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Do NOT use commas - some English meanings naturally contain commas.</t>
+          <t xml:space="preserve">   Row 4, Column A: Third passage text.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Example: park, garden|to like, prefer  &lt;- would break if using comma delimiter</t>
-        </is>
-      </c>
+      <c r="A52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>DELIMITER RULE (Vocabulary + English columns)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>MULTI-PRONUNCIATION CHARACTERS (多音字)</t>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Use | (pipe character) to separate items in Vocabulary and English columns.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Some Traditional Chinese characters have multiple pronunciations that pypinyin</t>
+          <t>Do NOT use commas - some English meanings naturally contain commas.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>may guess incorrectly. Common examples:</t>
+          <t>Example: park, garden|to like, prefer  &lt;- would break if using comma delimiter</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  長: cháng (long) vs zhǎng (elder/grow) - e.g., 長方形 should be cháng fāng xíng</t>
-        </is>
-      </c>
+      <c r="A57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  行: xíng (walk) vs háng (row/profession) - e.g., 銀行 = yín háng</t>
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>MULTI-PRONUNCIATION CHARACTERS (多音字)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">  樂: lè (happy) vs yuè (music) - e.g., 音樂 = yīn yuè</t>
+          <t>Some Traditional Chinese characters have multiple pronunciations that pypinyin</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
+        <is>
+          <t>may guess incorrectly. Common examples:</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  長: cháng (long) vs zhǎng (elder/grow) - e.g., 長方形 should be cháng fāng xíng</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  行: xíng (walk) vs háng (row/profession) - e.g., 銀行 = yín háng</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  樂: lè (happy) vs yuè (music) - e.g., 音樂 = yīn yuè</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>Fix these manually during the review step.</t>
         </is>

</xml_diff>